<commit_message>
Source dossier: correct the US import unit value band to 2025 quarterly totals
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FPeEPN6oNfciD5oEqditMq
</commit_message>
<xml_diff>
--- a/data/source_dossier.xlsx
+++ b/data/source_dossier.xlsx
@@ -1987,7 +1987,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Fig. A.1 technical-grade band 2.40–2.70 $/kg (US import unit value, CIF, 2025)</t>
+          <t>Fig. A.1 technical-grade band 2.43–2.55 $/kg (US import unit value of total hydrofluoric acid imports, CIF, 2025 quarters), shown as 2.4–2.6</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Total-row unit values span 2.43–2.55 $/kg in 2025 (2.47 for the year); the 2.70 upper end of the Fig. A.1 band is reached only at country level (e.g., Mexico, Q2 2025: 41,200/15,300 = 2.69 $/kg). State the basis of the band in the figure caption.</t>
+          <t>Total-row unit values span 2.43–2.55 $/kg in 2025 (2.47 for the year); the band was corrected from 2.4–2.7 on 2026-10-05.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Source dossier: align citation labels with the SI and cite the 2025 fluorspar review
- Citation labels now match the Supplementary Information: Business Society, 2025a/2025b;
  Kim, J.-U., 2026 (Dealsite) and Kim, J.-H., 2026 (Money Today).
- Business Society, 2025a now points to the 2025 fluorspar market review (Sina Finance,
  2025-12-30), which gives 3,622.5 CNY/t as the start-of-2025 average used as the upper bound
  of the fluorspar price range.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FPeEPN6oNfciD5oEqditMq
</commit_message>
<xml_diff>
--- a/data/source_dossier.xlsx
+++ b/data/source_dossier.xlsx
@@ -988,7 +988,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Business Society, 2025</t>
+          <t>Business Society, 2025b</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1273,7 +1273,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Kim, 2026</t>
+          <t>Kim, J.-U., 2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Reporter Kim Ji-hyun (distinct from 'Kim, 2026', the Dealsite article). 'Last year' = 2025; 'this month' = April 2026.</t>
+          <t>Reporter Kim Ji-hyun (distinct from 'Kim, J.-U., 2026', the Dealsite article). 'Last year' = 2025; 'this month' = April 2026.</t>
         </is>
       </c>
     </row>
@@ -2138,47 +2138,47 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>生意社：2024年氢氟酸行情回顾及2025年的展望</t>
+          <t>生意社：2025年萤石行情下滑 2026年将弱势复苏</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Review of the 2024 hydrofluoric acid market and outlook for 2025</t>
+          <t>Fluorspar prices fell in 2025 and are expected to recover weakly in 2026</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.100ppi.com/forecast/detail-20250113-197484.html</t>
+          <t>https://finance.sina.com.cn/money/future/nyzx/2025-12-30/doc-inheqixr5797475.shtml</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Paragraph on raw-material fluorspar (published 2025-01-13)</t>
+          <t>Paragraph on the 2025 fluorspar market (Business Society via Sina Finance, published 2025-12-30)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Fluorspar average price 3,531.25 CNY/t (start of 2024) and 3,622.5 CNY/t (end of 2024); 3,622.5 used as the 2025 start-of-year value</t>
+          <t>Fluorspar average price 3,622.5 CNY/t (start of 2025) and 3,400 CNY/t (end of 2025); 3,622.5 used as the upper bound of the fluorspar price range</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>在2024年，萤石价格呈现小幅上涨趋势，年初平均价格为3531.25元/吨，年底均价为3622.5元/吨，涨幅2.58%。</t>
+          <t>2025年国内萤石价格走势下滑，年初平均价格为3622.5元/吨，年底萤石均价为3400元/吨，全年跌幅为6.14%。</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>In 2024, fluorspar prices rose slightly: the average price was 3,531.25 CNY/t at the start of the year and 3,622.5 CNY/t at the end of the year, an increase of 2.58%.</t>
+          <t>Domestic fluorspar prices fell in 2025: the average price was 3,622.5 CNY/t at the start of the year and 3,400 CNY/t at the end of the year, a decrease of 6.14% over the year.</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>excerpt verified 2026-10-05</t>
+          <t>excerpt verified 2026-10-12</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>The source gives 3,622.5 CNY/t as the end-of-2024 average, not a 2025 value; using it as the 2025 start-of-year price is an interpretation. The page sits behind a browser check; text read after passing the check. If cited alongside 'Business Society, 2025' (rawmex), use 2025a/2025b.</t>
+          <t>Replaces the earlier entry (Business Society review of the 2024 market, 100ppi.com, 2025-01-13), which reports the same 3,622.5 CNY/t as the end-of-2024 average.</t>
         </is>
       </c>
     </row>

</xml_diff>